<commit_message>
docs(qa): expand AI Diagnosis BRD to full AC + Claude master prompt
Implementation-ready BRD §§1–14 with acceptance criteria for all 64
requirements, corrected Past Diagnoses scoring, 47 test scenarios, and
a paste-ready Claude Code MASTER PROMPT (Waves 0–4).

Co-authored-by: manojkparija <manojkparija@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/qa/diagnosis/GAADIIQ_AI_Diagnosis_BRD_QA.xlsx
+++ b/docs/qa/diagnosis/GAADIIQ_AI_Diagnosis_BRD_QA.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Executive" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Requirements" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="TestCases" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="AcceptanceCriteria" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -438,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,87 +457,99 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-25 13:53 UTC</t>
+          <t>2026-07-25 13:56 UTC</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BRD Score</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>63</v>
+          <t>Code tip</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>claude/gaadiiq-app-dev-abj5fo</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Req PASS</t>
+          <t>BRD Score</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>31</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Req PARTIAL</t>
+          <t>Req PASS</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Req FAIL</t>
+          <t>Req PARTIAL</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Test PASS</t>
+          <t>Req FAIL</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Test PARTIAL</t>
+          <t>Test PASS</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Test FAIL</t>
+          <t>Test PARTIAL</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Test FAIL</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Recommendation</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>NO-GO for full BRD; CONDITIONAL for manual+image MVP</t>
         </is>
@@ -553,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -592,6 +605,11 @@
           <t>Gap</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Justification</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -621,12 +639,17 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Angular Step 1 form</t>
+          <t>Angular Step 1 form (make/model/year/fuel/transmission)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Baseline path for users who prefer typing</t>
         </is>
       </c>
     </row>
@@ -658,12 +681,17 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>voice-mode overlay + STT</t>
+          <t>voice-mode overlay + Web Speech STT</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Hands-free capture for drivers / literacy barriers</t>
         </is>
       </c>
     </row>
@@ -695,12 +723,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>vehicle-info-extractor + /voice/extract</t>
+          <t>vehicle-info-extractor + POST /diagnosis/voice/extract</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Reduce form friction after speech</t>
         </is>
       </c>
     </row>
@@ -732,12 +765,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>onVoiceCompleted merges form</t>
+          <t>onVoiceCompleted merges into form signals</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Keep single source of truth for review step</t>
         </is>
       </c>
     </row>
@@ -769,12 +807,17 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>step1Valid + Pydantic</t>
+          <t>step1Valid + Pydantic DiagnoseRequest</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Prevent invalid analyse payloads</t>
         </is>
       </c>
     </row>
@@ -806,12 +849,17 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>voice-mode _askMissingFields</t>
+          <t>voice-mode _askMissingFields TTS loop</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Complete mandatory vehicle fields before analyse</t>
         </is>
       </c>
     </row>
@@ -843,12 +891,17 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Step 2 textarea</t>
+          <t>Step 2 textarea problem_description</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Primary symptom capture</t>
         </is>
       </c>
     </row>
@@ -880,12 +933,17 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Step 2 mic + overlay</t>
+          <t>Step 2 mic toolbar + overlay problem phase</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Speak symptoms in native language</t>
         </is>
       </c>
     </row>
@@ -917,12 +975,17 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>POST /upload/image</t>
+          <t>POST /upload/image → image_urls</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Visual context for vision + mechanic handoff</t>
         </is>
       </c>
     </row>
@@ -954,12 +1017,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Schema audio_url only</t>
+          <t>DB/schema audio_url exists; unused</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>No UI/API upload</t>
+          <t>No POST /upload/audio or Step 2 UI</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Engine noise / rattles improve diagnosis</t>
         </is>
       </c>
     </row>
@@ -991,12 +1059,17 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Schema video_url only</t>
+          <t>DB/schema video_url exists; unused</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>No video upload</t>
+          <t>No video upload API/UI</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Capture intermittent symptoms</t>
         </is>
       </c>
     </row>
@@ -1028,12 +1101,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>WARNING_LIGHTS chips</t>
+          <t>WARNING_LIGHTS chips in Step 2</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Structured symptom signals</t>
         </is>
       </c>
     </row>
@@ -1065,12 +1143,17 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Not in form/API</t>
+          <t>Not in form/API/model</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>No maintenance_history field</t>
+          <t>Add maintenance_history JSON field</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Prior service context</t>
         </is>
       </c>
     </row>
@@ -1102,12 +1185,17 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>detectLanguageFromText unwired</t>
+          <t>detectLanguageFromText exists client-side</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Wire autoDetect into voice session</t>
+          <t>Wire Auto-detect toggle into voice session</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Users may not know BCP-47 codes</t>
         </is>
       </c>
     </row>
@@ -1139,12 +1227,17 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>11 VOICE_LANGUAGES</t>
+          <t>11 VOICE_LANGUAGES in picker</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Prompts fully localized for 6 only</t>
+          <t>PROMPTS fully localized for 6 only</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>India language coverage</t>
         </is>
       </c>
     </row>
@@ -1184,6 +1277,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Consistent journey language</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1218,7 +1316,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Quality untested; may stay EN</t>
+          <t>Golden-set QA; English fallback banner</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Trust for non-English users</t>
         </is>
       </c>
     </row>
@@ -1250,12 +1353,17 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Browser Web Speech only</t>
+          <t>Browser Web Speech API only</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>No server STT; WebView risk</t>
+          <t>Server STT + MediaRecorder for WebView</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Production Android/iOS reliability</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1400,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>No server TTS</t>
+          <t>Optional server TTS; keep client fallback</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Playback on devices with weak voices</t>
         </is>
       </c>
     </row>
@@ -1324,12 +1437,17 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>interimText UI</t>
+          <t>interimText in voice overlay</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>User confidence while speaking</t>
         </is>
       </c>
     </row>
@@ -1369,6 +1487,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Listen to diagnosis</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1398,12 +1521,17 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>replaySpeaking</t>
+          <t>replaySpeaking()</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Re-hear instructions</t>
         </is>
       </c>
     </row>
@@ -1435,12 +1563,17 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>pauseSpeaking</t>
+          <t>pauseSpeaking()</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Interruptible playback</t>
         </is>
       </c>
     </row>
@@ -1472,12 +1605,17 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>stop STT/TTS</t>
+          <t>stop STT/TTS controls</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Immediate silence</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1652,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>No always-on driving mode</t>
+          <t>Always-on driving mode</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Parked/driving safety</t>
         </is>
       </c>
     </row>
@@ -1546,12 +1689,17 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Large overlay</t>
+          <t>Large overlay UI</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>No driving mode; RECORD_AUDIO gap</t>
+          <t>Driving mode + RECORD_AUDIO</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Large targets, reduced glances</t>
         </is>
       </c>
     </row>
@@ -1583,12 +1731,17 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>services/diagnosis.py</t>
+          <t>services/diagnosis.py run_diagnosis</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Primary LLM path</t>
         </is>
       </c>
     </row>
@@ -1620,12 +1773,17 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Keyword KB 12 cases</t>
+          <t>Keyword match on repair_knowledge.json (12 cases)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Not vector RAG for diagnosis</t>
+          <t>Vector RAG over KB (Qdrant/BGE unused)</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Grounded repair advice</t>
         </is>
       </c>
     </row>
@@ -1665,6 +1823,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Core diagnosis value</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1702,6 +1865,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Urgency signalling</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1731,12 +1899,17 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>safe_to_drive UI</t>
+          <t>safe_to_drive + UI warning</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Safety-critical output</t>
         </is>
       </c>
     </row>
@@ -1768,12 +1941,17 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>cost_min/max INR</t>
+          <t>cost_min_inr / cost_max_inr</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Budget transparency</t>
         </is>
       </c>
     </row>
@@ -1813,6 +1991,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Time planning</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1842,12 +2025,17 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>recommended_steps + DIY</t>
+          <t>recommended_steps + How to Fix</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Actionable guidance</t>
         </is>
       </c>
     </row>
@@ -1887,6 +2075,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Upsell prevention</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1921,7 +2114,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>No post-diagnosis follow-ups</t>
+          <t>Post-diagnosis follow_up_questions[]</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Improve low-confidence cases</t>
         </is>
       </c>
     </row>
@@ -1953,12 +2151,17 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Responsive SCSS</t>
+          <t>Responsive SCSS + layout e2e</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Not dedicated mobile shell</t>
+          <t>Dedicated mobile shell polish</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Primary usage is phone</t>
         </is>
       </c>
     </row>
@@ -1990,12 +2193,17 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Steps 1–3</t>
+          <t>Steps 1–3 wizard progress</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Orient user in flow</t>
         </is>
       </c>
     </row>
@@ -2027,12 +2235,17 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>In-session + API history</t>
+          <t>Past Diagnoses panel + GET /history</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>No Angular history UI / conversation DB</t>
+          <t>No multi-turn conversation DB/UI; open-by-id weak</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Revisit prior advice</t>
         </is>
       </c>
     </row>
@@ -2072,6 +2285,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>User preference</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2101,12 +2319,17 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>STT + diag error cards</t>
+          <t>STT + diagnosis error cards</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Recoverable failures</t>
         </is>
       </c>
     </row>
@@ -2138,12 +2361,17 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>clientFallback</t>
+          <t>clientFallback when API down</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Web Speech needs network</t>
+          <t>Offline banner; STT needs network</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Low-connectivity India</t>
         </is>
       </c>
     </row>
@@ -2175,12 +2403,17 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Browser not-allowed string</t>
+          <t>Browser not-allowed string only</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Android RECORD_AUDIO + consent UX</t>
+          <t>Android RECORD_AUDIO + Capacitor helper</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>OS-level mic access</t>
         </is>
       </c>
     </row>
@@ -2212,12 +2445,17 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>TLS assumed</t>
+          <t>TLS in transit assumed</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>No recording at-rest design</t>
+          <t>At-rest encryption design for recordings</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Protect voice PII</t>
         </is>
       </c>
     </row>
@@ -2249,12 +2487,17 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Postgres + R2 images</t>
+          <t>Postgres + R2 for images</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Transcripts not stored</t>
+          <t>Transcripts not stored securely</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Controlled retention</t>
         </is>
       </c>
     </row>
@@ -2286,12 +2529,17 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Generic privacy only</t>
+          <t>Generic privacy pages only</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>No mic consent gate</t>
+          <t>Pre-STT consent modal (purpose/retention)</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>DPDP / lawful processing</t>
         </is>
       </c>
     </row>
@@ -2323,12 +2571,17 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Nothing persisted</t>
+          <t>Nothing voice-persisted yet</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Need retention + delete API</t>
+          <t>Retention + DELETE voice APIs</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>User control of biometric-adjacent data</t>
         </is>
       </c>
     </row>
@@ -2360,12 +2613,17 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Disclaimer pages</t>
+          <t>Disclaimer copy</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>No diagnosis delete UX</t>
+          <t>Diagnosis/voice delete UX</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>India DPDP Act readiness</t>
         </is>
       </c>
     </row>
@@ -2397,12 +2655,17 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Fallback fast</t>
+          <t>Heuristic fallback fast</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Ollama unbounded</t>
+          <t>Ollama timeout ≤8s → fallback</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Perceived performance</t>
         </is>
       </c>
     </row>
@@ -2434,12 +2697,17 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Browser STT + retry</t>
+          <t>Browser STT + noisy retry</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>No benchmarks</t>
+          <t>WER benchmarks per language</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Voice trust</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2744,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>No golden-set tests</t>
+          <t>Golden-set fixtures in CI</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Safety + usefulness</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2786,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>POST /diagnosis/stt needed</t>
+          <t>POST /diagnosis/stt (multipart)</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>WebView production path</t>
         </is>
       </c>
     </row>
@@ -2550,7 +2828,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Server TTS optional</t>
+          <t>POST /diagnosis/tts optional</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Consistent voice quality</t>
         </is>
       </c>
     </row>
@@ -2582,12 +2865,17 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Client-only</t>
+          <t>Client-only heuristic</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
           <t>POST /diagnosis/detect-language</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Server-side lang detect</t>
         </is>
       </c>
     </row>
@@ -2619,12 +2907,17 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Internal translate</t>
+          <t>Internal _translate_diagnosis</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Not standalone</t>
+          <t>Not standalone endpoint</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Reuse across modules</t>
         </is>
       </c>
     </row>
@@ -2664,6 +2957,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Core backend</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2701,6 +2999,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Media pipeline</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2738,6 +3041,11 @@
           <t>POST /upload/audio</t>
         </is>
       </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Persist engine audio</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2772,7 +3080,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>voice_transcripts table</t>
+          <t>voice_transcripts (consent-gated)</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Audit + improve STT</t>
         </is>
       </c>
     </row>
@@ -2804,12 +3117,17 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>In-memory only</t>
+          <t>In-session memory only</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
           <t>diagnosis_conversations</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Multi-turn persistence</t>
         </is>
       </c>
     </row>
@@ -2841,12 +3159,17 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>vehicle_diagnoses</t>
+          <t>vehicle_diagnoses + Past Diagnoses UI</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Angular history UI gap</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>User revisit</t>
         </is>
       </c>
     </row>
@@ -2886,6 +3209,11 @@
           <t>diagnosis_audit_events</t>
         </is>
       </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Compliance + debug</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2915,12 +3243,17 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>No test_diagnosis.py</t>
+          <t>No test_diagnosis.py / extractor specs</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Critical QA gap</t>
+          <t>Add pytest + unit tests</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Prevent regressions</t>
         </is>
       </c>
     </row>
@@ -2952,12 +3285,17 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Manifest gap for mic</t>
+          <t>Manifest has CAMERA/location only</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Add permission + plugin</t>
+          <t>Add RECORD_AUDIO + runtime request</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>APK mic required</t>
         </is>
       </c>
     </row>
@@ -2972,7 +3310,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3532,22 +3870,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Angular diagnosis history UI</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Angular Past Diagnoses history UI</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>API only</t>
+          <t>history-panel on Claude tip</t>
         </is>
       </c>
     </row>
@@ -3778,81 +4116,81 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>TC-S-01</t>
+          <t>TC-F-25</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Unauth GET diagnosis denied</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>Open past diagnosis by id from history</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>owner auth</t>
+          <t>List only; no detail navigation</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>TC-S-02</t>
+          <t>TC-F-26</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Prompt injection fencing</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+          <t>Guest can analyse without login</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>User text in prompts</t>
+          <t>Public analyse + rate limit</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>TC-S-03</t>
+          <t>TC-F-27</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Rate limit analyse</t>
+          <t>detected_language sent on analyse</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -3867,7 +4205,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>documented limits</t>
+          <t>Claude Angular + DiagnoseRequest</t>
         </is>
       </c>
     </row>
@@ -3879,44 +4217,44 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>TC-S-04</t>
+          <t>TC-S-01</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Audio upload validation</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Unauth GET diagnosis denied</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>No audio upload</t>
+          <t>owner auth</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>TC-P-01</t>
+          <t>TC-S-02</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Analyse p95 with fallback</t>
+          <t>Prompt injection fencing</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -3926,125 +4264,125 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Ollama unbounded</t>
+          <t>User text in prompts</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>TC-P-02</t>
+          <t>TC-S-03</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>STT works offline</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Rate limit analyse</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Web Speech needs net</t>
+          <t>documented limits</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>A11y</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>TC-A-01</t>
+          <t>TC-S-04</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Voice overlay SR labels</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+          <t>Audio upload validation</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Audit incomplete</t>
+          <t>No audio upload</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>TC-M-01</t>
+          <t>TC-S-05</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>No horizontal overflow on route</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>Mic consent logged before STT</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>mobile-layout e2e</t>
+          <t>No consent event</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>TC-M-02</t>
+          <t>TC-P-01</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Voice overlay one-handed</t>
+          <t>Analyse p95 with fallback</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -4054,29 +4392,29 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>No driving mode</t>
+          <t>Ollama unbounded</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Regression</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>TC-R-01</t>
+          <t>TC-P-02</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>API pytest diagnosis suite</t>
+          <t>STT works offline</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -4086,98 +4424,98 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>No test_diagnosis.py</t>
+          <t>Web Speech needs net</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Regression</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>TC-R-02</t>
+          <t>TC-P-03</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Voice extractor unit tests</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>Image upload ≤10MB reject</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>No *.spec.ts</t>
+          <t>upload validation path</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>A11y</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>TC-I-01</t>
+          <t>TC-A-01</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Ollama down → heuristic report</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>Voice overlay SR labels</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>fallback path</t>
+          <t>Audit incomplete</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>A11y</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TC-I-02</t>
+          <t>TC-A-02</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Vision on image_url</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+          <t>aria-live for interim transcript</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -4187,24 +4525,24 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>vision.py untested quality</t>
+          <t>Missing</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Usability</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TC-U-01</t>
+          <t>TC-M-01</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Manual vs Voice mode clear</t>
+          <t>No horizontal overflow on route</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -4219,39 +4557,1414 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Step 1 selector</t>
+          <t>mobile-layout e2e</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>TC-M-02</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Voice overlay one-handed</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>No driving mode</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>TC-R-01</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>API pytest diagnosis suite</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>No test_diagnosis.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TC-R-02</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Voice extractor unit tests</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>No *.spec.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>TC-I-01</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Ollama down → heuristic report</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>fallback path</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>TC-I-02</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Vision on image_url</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>vision.py untested quality</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>TC-I-03</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>voice/extract then autofill</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Claude tip path</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>Usability</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>TC-U-01</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Manual vs Voice mode clear</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Step 1 selector</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Usability</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
         <is>
           <t>TC-U-02</t>
         </is>
       </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Disclaimer before submit</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Step 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Usability</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>TC-U-03</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>safe_to_drive=false banner prominence</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Report warning UI</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C65"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Requirement ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BR-VI-01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Manual vehicle entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BR-VI-02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Voice vehicle entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BR-VI-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Auto-extract from speech</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BR-VI-04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Auto-fill form</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BR-VI-05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Intelligent validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BR-VI-06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Missing info prompts</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BR-IR-01</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Text issue report</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BR-IR-02</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Voice issue report</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BR-IR-03</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Image upload</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BR-IR-04</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Audio upload</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BR-IR-05</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Video upload</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BR-IR-06</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Warning lights</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BR-IR-07</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Maintenance history</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BR-ML-01</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Auto language detect</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BR-ML-02</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Indian languages</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BR-ML-03</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Preserve language</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BR-ML-04</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>AI language match</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BR-VA-01</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BR-VA-02</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>TTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BR-VA-03</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Live transcription</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BR-VA-04</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Voice playback</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BR-VA-05</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Replay</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>BR-VA-06</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Pause</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>BR-VA-07</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>BR-VA-08</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Hands-free</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>BR-VA-09</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Driver-friendly</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>BR-AI-01</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Ollama</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>BR-AI-02</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>RAG KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>BR-AI-03</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Root cause</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>BR-AI-04</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>BR-AI-05</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Safe-to-drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>BR-AI-06</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Repair cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BR-AI-07</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Repair duration</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>BR-AI-08</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Next steps</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>BR-AI-09</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Preventive</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>BR-AI-10</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Follow-ups</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>BR-UX-01</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Mobile-first</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>BR-UX-02</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>BR-UX-03</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Disclaimer before submit</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Step 3</t>
+          <t>Conversation history</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>BR-UX-04</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Voice/Text switch</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>BR-UX-05</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Error handling</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>BR-UX-06</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>BR-SEC-01</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Mic permissions</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>BR-SEC-02</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Voice encryption</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>BR-SEC-03</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Secure storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>BR-SEC-04</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Mic consent</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>BR-SEC-05</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Delete recordings</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>BR-SEC-06</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>DPDP</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>BR-PERF-01</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Fast response</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>BR-PERF-02</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>STT accuracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>BR-PERF-03</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>AI accuracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>BR-API-01</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>STT API</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>BR-API-02</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>TTS API</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>BR-API-03</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Lang detect API</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>BR-API-04</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Translation API</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>BR-API-05</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Diagnosis API</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>BR-API-06</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Image upload API</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>BR-API-07</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Audio upload API</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>BR-DB-01</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Transcript storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>BR-DB-02</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Conversation storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>BR-DB-03</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Diagnosis history</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>BR-DB-04</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Audit logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>BR-TEST-01</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Automated tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>BR-AND-01</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Android RECORD_AUDIO</t>
         </is>
       </c>
     </row>

</xml_diff>